<commit_message>
JTAI refresh, 2026-05-18 06:28:38
</commit_message>
<xml_diff>
--- a/ofsted_csc_jtai_overview.xlsx
+++ b/ofsted_csc_jtai_overview.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="817" uniqueCount="548">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="558">
   <si>
     <t>80426</t>
   </si>
@@ -1400,6 +1400,36 @@
   </si>
   <si>
     <t>The effectiveness of management oversight and supervision across health and police services. Management and staff capacity in the police, early help teams and health services. The timely provision of suitable accommodation for children subject to police protection.</t>
+  </si>
+  <si>
+    <t>80516</t>
+  </si>
+  <si>
+    <t>211</t>
+  </si>
+  <si>
+    <t>E09000030</t>
+  </si>
+  <si>
+    <t>204, 206, 316, 352, 202, 309, 213, 210, 330, 304</t>
+  </si>
+  <si>
+    <t>tower hamlets</t>
+  </si>
+  <si>
+    <t>https://files.ofsted.gov.uk/v1/file/50301682</t>
+  </si>
+  <si>
+    <t>14/05/26</t>
+  </si>
+  <si>
+    <t>Child sexual abuse in the family environment in tower hamlets.</t>
+  </si>
+  <si>
+    <t>Tower Hamlets is a London borough that is characterised by a rich mix of cultural diversity, with many families who speak English as an additional language and are disproportionately affected by poverty, overcrowding and inequality. Agencies across the partnership have good awareness of this and it is typically addressed in their 2 practice. Across the partnership, joint working and communication are strong, resulting in effective, collaborative, child-centred practice for most children in the borough.</t>
+  </si>
+  <si>
+    <t>The professional curiosity of staff across agencies, especially in circumstances where children are not consistently believed by some families or there are multiple vulnerabilities present, such as domestic abuse, coercion, and control and neglect. The consistent quality and effectiveness of safety plans and assessments. The consistency and timely distribution of the minutes and agreed actions from child protection strategy meetings to relevant partner agencies.</t>
   </si>
   <si>
     <t>80521</t>
@@ -2020,63 +2050,63 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R48"/>
+  <dimension ref="A1:R49"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
       <c r="A1" s="1" t="s">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>531</v>
+        <v>541</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>532</v>
+        <v>542</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>533</v>
+        <v>543</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>534</v>
+        <v>544</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>535</v>
+        <v>545</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>536</v>
+        <v>546</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>537</v>
+        <v>547</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>538</v>
+        <v>548</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>539</v>
+        <v>549</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>540</v>
+        <v>550</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>541</v>
+        <v>551</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>542</v>
+        <v>552</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>543</v>
+        <v>553</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>544</v>
+        <v>554</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>545</v>
+        <v>555</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>546</v>
+        <v>556</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>547</v>
+        <v>557</v>
       </c>
     </row>
     <row r="2" spans="1:18">
@@ -4424,7 +4454,7 @@
         <v>463</v>
       </c>
       <c r="C43" t="s">
-        <v>27</v>
+        <v>321</v>
       </c>
       <c r="D43" t="s">
         <v>464</v>
@@ -4445,7 +4475,7 @@
         <v>468</v>
       </c>
       <c r="J43" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80521_manchester", ".\export_data\inspection_reports\80521_manchester")</f>
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80516_tower hamlets", ".\export_data\inspection_reports\80516_tower hamlets")</f>
         <v>0</v>
       </c>
       <c r="K43" t="s">
@@ -4458,13 +4488,13 @@
         <v>9</v>
       </c>
       <c r="N43" t="s">
+        <v>68</v>
+      </c>
+      <c r="O43" t="s">
         <v>470</v>
       </c>
-      <c r="O43" t="s">
+      <c r="P43" t="s">
         <v>471</v>
-      </c>
-      <c r="P43" t="s">
-        <v>472</v>
       </c>
       <c r="Q43" t="s">
         <v>12</v>
@@ -4475,224 +4505,224 @@
     </row>
     <row r="44" spans="1:18">
       <c r="A44" t="s">
+        <v>472</v>
+      </c>
+      <c r="B44" t="s">
         <v>473</v>
       </c>
-      <c r="B44" t="s">
+      <c r="C44" t="s">
+        <v>27</v>
+      </c>
+      <c r="D44" t="s">
         <v>474</v>
       </c>
-      <c r="C44" t="s">
+      <c r="E44" t="s">
         <v>475</v>
       </c>
-      <c r="D44" t="s">
+      <c r="F44" t="s">
         <v>476</v>
       </c>
-      <c r="E44" t="s">
+      <c r="G44" s="2" t="s">
         <v>477</v>
       </c>
-      <c r="F44" t="s">
+      <c r="H44" t="s">
         <v>478</v>
       </c>
-      <c r="G44" s="2" t="s">
+      <c r="I44" t="s">
+        <v>478</v>
+      </c>
+      <c r="J44" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80521_manchester", ".\export_data\inspection_reports\80521_manchester")</f>
+        <v>0</v>
+      </c>
+      <c r="K44" t="s">
         <v>479</v>
       </c>
-      <c r="H44" t="s">
+      <c r="L44" t="s">
+        <v>9</v>
+      </c>
+      <c r="M44" t="s">
+        <v>9</v>
+      </c>
+      <c r="N44" t="s">
         <v>480</v>
       </c>
-      <c r="I44" t="s">
-        <v>480</v>
-      </c>
-      <c r="J44" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80522_medway", ".\export_data\inspection_reports\80522_medway")</f>
-        <v>0</v>
-      </c>
-      <c r="K44" t="s">
+      <c r="O44" t="s">
         <v>481</v>
       </c>
-      <c r="L44" t="s">
-        <v>9</v>
-      </c>
-      <c r="M44" t="s">
+      <c r="P44" t="s">
         <v>482</v>
       </c>
-      <c r="N44" t="s">
-        <v>483</v>
-      </c>
-      <c r="O44" t="s">
-        <v>9</v>
-      </c>
-      <c r="P44" t="s">
-        <v>9</v>
-      </c>
       <c r="Q44" t="s">
-        <v>484</v>
+        <v>12</v>
       </c>
       <c r="R44" t="s">
-        <v>485</v>
+        <v>9</v>
       </c>
     </row>
     <row r="45" spans="1:18">
       <c r="A45" t="s">
+        <v>483</v>
+      </c>
+      <c r="B45" t="s">
+        <v>484</v>
+      </c>
+      <c r="C45" t="s">
+        <v>485</v>
+      </c>
+      <c r="D45" t="s">
         <v>486</v>
       </c>
-      <c r="B45" t="s">
+      <c r="E45" t="s">
         <v>487</v>
       </c>
-      <c r="C45" t="s">
-        <v>50</v>
-      </c>
-      <c r="D45" t="s">
+      <c r="F45" t="s">
         <v>488</v>
       </c>
-      <c r="E45" t="s">
+      <c r="G45" s="2" t="s">
         <v>489</v>
       </c>
-      <c r="F45" t="s">
+      <c r="H45" t="s">
         <v>490</v>
       </c>
-      <c r="G45" s="2" t="s">
+      <c r="I45" t="s">
+        <v>490</v>
+      </c>
+      <c r="J45" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80522_medway", ".\export_data\inspection_reports\80522_medway")</f>
+        <v>0</v>
+      </c>
+      <c r="K45" t="s">
         <v>491</v>
       </c>
-      <c r="H45" t="s">
+      <c r="L45" t="s">
+        <v>9</v>
+      </c>
+      <c r="M45" t="s">
         <v>492</v>
       </c>
-      <c r="I45" t="s">
-        <v>492</v>
-      </c>
-      <c r="J45" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80524_milton keynes", ".\export_data\inspection_reports\80524_milton keynes")</f>
-        <v>0</v>
-      </c>
-      <c r="K45" t="s">
+      <c r="N45" t="s">
         <v>493</v>
       </c>
-      <c r="L45" t="s">
-        <v>9</v>
-      </c>
-      <c r="M45" t="s">
+      <c r="O45" t="s">
+        <v>9</v>
+      </c>
+      <c r="P45" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q45" t="s">
         <v>494</v>
       </c>
-      <c r="N45" t="s">
+      <c r="R45" t="s">
         <v>495</v>
-      </c>
-      <c r="O45" t="s">
-        <v>9</v>
-      </c>
-      <c r="P45" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q45" t="s">
-        <v>82</v>
-      </c>
-      <c r="R45" t="s">
-        <v>496</v>
       </c>
     </row>
     <row r="46" spans="1:18">
       <c r="A46" t="s">
+        <v>496</v>
+      </c>
+      <c r="B46" t="s">
         <v>497</v>
       </c>
-      <c r="B46" t="s">
+      <c r="C46" t="s">
+        <v>50</v>
+      </c>
+      <c r="D46" t="s">
         <v>498</v>
       </c>
-      <c r="C46" t="s">
-        <v>15</v>
-      </c>
-      <c r="D46" t="s">
+      <c r="E46" t="s">
         <v>499</v>
       </c>
-      <c r="E46" t="s">
+      <c r="F46" t="s">
         <v>500</v>
       </c>
-      <c r="F46" t="s">
+      <c r="G46" s="2" t="s">
         <v>501</v>
       </c>
-      <c r="G46" s="2" t="s">
+      <c r="H46" t="s">
         <v>502</v>
       </c>
-      <c r="H46" t="s">
+      <c r="I46" t="s">
+        <v>502</v>
+      </c>
+      <c r="J46" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80524_milton keynes", ".\export_data\inspection_reports\80524_milton keynes")</f>
+        <v>0</v>
+      </c>
+      <c r="K46" t="s">
         <v>503</v>
       </c>
-      <c r="I46" t="s">
-        <v>503</v>
-      </c>
-      <c r="J46" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80418_norfolk", ".\export_data\inspection_reports\80418_norfolk")</f>
-        <v>0</v>
-      </c>
-      <c r="K46" t="s">
+      <c r="L46" t="s">
+        <v>9</v>
+      </c>
+      <c r="M46" t="s">
         <v>504</v>
-      </c>
-      <c r="L46" t="s">
-        <v>9</v>
-      </c>
-      <c r="M46" t="s">
-        <v>9</v>
       </c>
       <c r="N46" t="s">
         <v>505</v>
       </c>
       <c r="O46" t="s">
+        <v>9</v>
+      </c>
+      <c r="P46" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q46" t="s">
+        <v>82</v>
+      </c>
+      <c r="R46" t="s">
         <v>506</v>
-      </c>
-      <c r="P46" t="s">
-        <v>507</v>
-      </c>
-      <c r="Q46" t="s">
-        <v>12</v>
-      </c>
-      <c r="R46" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="47" spans="1:18">
       <c r="A47" t="s">
+        <v>507</v>
+      </c>
+      <c r="B47" t="s">
         <v>508</v>
       </c>
-      <c r="B47" t="s">
+      <c r="C47" t="s">
+        <v>15</v>
+      </c>
+      <c r="D47" t="s">
         <v>509</v>
       </c>
-      <c r="C47" t="s">
-        <v>2</v>
-      </c>
-      <c r="D47" t="s">
+      <c r="E47" t="s">
         <v>510</v>
       </c>
-      <c r="E47" t="s">
+      <c r="F47" t="s">
         <v>511</v>
       </c>
-      <c r="F47" t="s">
+      <c r="G47" s="2" t="s">
         <v>512</v>
       </c>
-      <c r="G47" s="2" t="s">
+      <c r="H47" t="s">
         <v>513</v>
       </c>
-      <c r="H47" t="s">
+      <c r="I47" t="s">
+        <v>513</v>
+      </c>
+      <c r="J47" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80418_norfolk", ".\export_data\inspection_reports\80418_norfolk")</f>
+        <v>0</v>
+      </c>
+      <c r="K47" t="s">
         <v>514</v>
       </c>
-      <c r="I47" t="s">
-        <v>514</v>
-      </c>
-      <c r="J47" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80530_north yorkshire", ".\export_data\inspection_reports\80530_north yorkshire")</f>
-        <v>0</v>
-      </c>
-      <c r="K47" t="s">
+      <c r="L47" t="s">
+        <v>9</v>
+      </c>
+      <c r="M47" t="s">
+        <v>9</v>
+      </c>
+      <c r="N47" t="s">
         <v>515</v>
       </c>
-      <c r="L47" t="s">
-        <v>9</v>
-      </c>
-      <c r="M47" t="s">
-        <v>9</v>
-      </c>
-      <c r="N47" t="s">
+      <c r="O47" t="s">
         <v>516</v>
       </c>
-      <c r="O47" t="s">
+      <c r="P47" t="s">
         <v>517</v>
-      </c>
-      <c r="P47" t="s">
-        <v>518</v>
       </c>
       <c r="Q47" t="s">
         <v>12</v>
@@ -4703,59 +4733,116 @@
     </row>
     <row r="48" spans="1:18">
       <c r="A48" t="s">
+        <v>518</v>
+      </c>
+      <c r="B48" t="s">
         <v>519</v>
       </c>
-      <c r="B48" t="s">
+      <c r="C48" t="s">
+        <v>2</v>
+      </c>
+      <c r="D48" t="s">
         <v>520</v>
       </c>
-      <c r="C48" t="s">
+      <c r="E48" t="s">
+        <v>521</v>
+      </c>
+      <c r="F48" t="s">
+        <v>522</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="H48" t="s">
+        <v>524</v>
+      </c>
+      <c r="I48" t="s">
+        <v>524</v>
+      </c>
+      <c r="J48" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80530_north yorkshire", ".\export_data\inspection_reports\80530_north yorkshire")</f>
+        <v>0</v>
+      </c>
+      <c r="K48" t="s">
+        <v>525</v>
+      </c>
+      <c r="L48" t="s">
+        <v>9</v>
+      </c>
+      <c r="M48" t="s">
+        <v>9</v>
+      </c>
+      <c r="N48" t="s">
+        <v>526</v>
+      </c>
+      <c r="O48" t="s">
+        <v>527</v>
+      </c>
+      <c r="P48" t="s">
+        <v>528</v>
+      </c>
+      <c r="Q48" t="s">
+        <v>12</v>
+      </c>
+      <c r="R48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:18">
+      <c r="A49" t="s">
+        <v>529</v>
+      </c>
+      <c r="B49" t="s">
+        <v>530</v>
+      </c>
+      <c r="C49" t="s">
         <v>185</v>
       </c>
-      <c r="D48" t="s">
-        <v>521</v>
-      </c>
-      <c r="E48" t="s">
-        <v>522</v>
-      </c>
-      <c r="F48" t="s">
-        <v>523</v>
-      </c>
-      <c r="G48" s="2" t="s">
-        <v>524</v>
-      </c>
-      <c r="H48" t="s">
-        <v>525</v>
-      </c>
-      <c r="I48" t="s">
-        <v>525</v>
-      </c>
-      <c r="J48" s="3">
+      <c r="D49" t="s">
+        <v>531</v>
+      </c>
+      <c r="E49" t="s">
+        <v>532</v>
+      </c>
+      <c r="F49" t="s">
+        <v>533</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="H49" t="s">
+        <v>535</v>
+      </c>
+      <c r="I49" t="s">
+        <v>535</v>
+      </c>
+      <c r="J49" s="3">
         <f>HYPERLINK(".\.\export_data\inspection_reports\80532_northumberland", ".\export_data\inspection_reports\80532_northumberland")</f>
         <v>0</v>
       </c>
-      <c r="K48" t="s">
-        <v>526</v>
-      </c>
-      <c r="L48" t="s">
-        <v>9</v>
-      </c>
-      <c r="M48" t="s">
-        <v>527</v>
-      </c>
-      <c r="N48" t="s">
-        <v>528</v>
-      </c>
-      <c r="O48" t="s">
-        <v>9</v>
-      </c>
-      <c r="P48" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q48" t="s">
+      <c r="K49" t="s">
+        <v>536</v>
+      </c>
+      <c r="L49" t="s">
+        <v>9</v>
+      </c>
+      <c r="M49" t="s">
+        <v>537</v>
+      </c>
+      <c r="N49" t="s">
+        <v>538</v>
+      </c>
+      <c r="O49" t="s">
+        <v>9</v>
+      </c>
+      <c r="P49" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q49" t="s">
         <v>82</v>
       </c>
-      <c r="R48" t="s">
-        <v>529</v>
+      <c r="R49" t="s">
+        <v>539</v>
       </c>
     </row>
   </sheetData>
@@ -4807,6 +4894,7 @@
     <hyperlink ref="G46" r:id="rId45"/>
     <hyperlink ref="G47" r:id="rId46"/>
     <hyperlink ref="G48" r:id="rId47"/>
+    <hyperlink ref="G49" r:id="rId48"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
JTAI refresh, 2026-05-25 06:32:57
</commit_message>
<xml_diff>
--- a/ofsted_csc_jtai_overview.xlsx
+++ b/ofsted_csc_jtai_overview.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="558">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="851" uniqueCount="568">
   <si>
     <t>80426</t>
   </si>
@@ -632,6 +632,36 @@
   </si>
   <si>
     <t>Children benefit from well-coordinated multi-agency working that is informed by high-quality assessments of needs completed and shared across relevant agencies in East Sussex. For one child, an exemplary quality health assessment resulted in prompt action to address undiagnosed and emerging emotional well-being and mental ill health needs. The contribution from a consultant paediatrician ensured a good understanding of the difficulties linked to the childs attention and hyperactivity disorder.</t>
+  </si>
+  <si>
+    <t>80469</t>
+  </si>
+  <si>
+    <t>390</t>
+  </si>
+  <si>
+    <t>E08000037</t>
+  </si>
+  <si>
+    <t>841, 357, 393, 372, 808, 840, 807, 394, 332, 384</t>
+  </si>
+  <si>
+    <t>gateshead</t>
+  </si>
+  <si>
+    <t>https://files.ofsted.gov.uk/v1/file/50302052</t>
+  </si>
+  <si>
+    <t>18/05/26</t>
+  </si>
+  <si>
+    <t>Child sexual abuse in the family environment in gateshead.</t>
+  </si>
+  <si>
+    <t>A mature, committed and professional partnership is working together to strengthen understanding and deliver continuous improvement to respond effectively to child sexual abuse in the family environment. The partnership has embedded a reflective and collaborative learning culture led by a trusted and effective chair of Gateshead multi-agency safeguarding arrangements (MASA). They work sensitively with community groups so that safeguarding and child sexual abuse are understood and integrated into the teaching children receive.</t>
+  </si>
+  <si>
+    <t>The development of a comprehensive partnership dataset to assist agencies understanding of the prevalence and profile of child sexual abuse in the family environment. Information-sharing at the front door that supports initial identification and assessment of risk across and within partner agencies. The consistent timeliness, attendance and recording of strategy meetings to enable multi-agency agreement of thresholds and shared decision-making of next steps, including joint investigations at the earliest opportunity.</t>
   </si>
   <si>
     <t>80470</t>
@@ -2050,63 +2080,63 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R49"/>
+  <dimension ref="A1:R50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
       <c r="A1" s="1" t="s">
-        <v>540</v>
+        <v>550</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>541</v>
+        <v>551</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>542</v>
+        <v>552</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>543</v>
+        <v>553</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>544</v>
+        <v>554</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>545</v>
+        <v>555</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>546</v>
+        <v>556</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>547</v>
+        <v>557</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>548</v>
+        <v>558</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>549</v>
+        <v>559</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>550</v>
+        <v>560</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>551</v>
+        <v>561</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>552</v>
+        <v>562</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>553</v>
+        <v>563</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>554</v>
+        <v>564</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>555</v>
+        <v>565</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>556</v>
+        <v>566</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>557</v>
+        <v>567</v>
       </c>
     </row>
     <row r="2" spans="1:18">
@@ -3143,7 +3173,7 @@
         <v>207</v>
       </c>
       <c r="C20" t="s">
-        <v>73</v>
+        <v>185</v>
       </c>
       <c r="D20" t="s">
         <v>208</v>
@@ -3164,7 +3194,7 @@
         <v>212</v>
       </c>
       <c r="J20" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80470_gloucestershire", ".\export_data\inspection_reports\80470_gloucestershire")</f>
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80469_gateshead", ".\export_data\inspection_reports\80469_gateshead")</f>
         <v>0</v>
       </c>
       <c r="K20" t="s">
@@ -3177,13 +3207,13 @@
         <v>9</v>
       </c>
       <c r="N20" t="s">
+        <v>68</v>
+      </c>
+      <c r="O20" t="s">
         <v>214</v>
       </c>
-      <c r="O20" t="s">
+      <c r="P20" t="s">
         <v>215</v>
-      </c>
-      <c r="P20" t="s">
-        <v>216</v>
       </c>
       <c r="Q20" t="s">
         <v>12</v>
@@ -3194,104 +3224,104 @@
     </row>
     <row r="21" spans="1:18">
       <c r="A21" t="s">
+        <v>216</v>
+      </c>
+      <c r="B21" t="s">
         <v>217</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
+        <v>73</v>
+      </c>
+      <c r="D21" t="s">
         <v>218</v>
       </c>
-      <c r="C21" t="s">
-        <v>27</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>219</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>220</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="G21" s="2" t="s">
+      <c r="H21" t="s">
         <v>222</v>
       </c>
-      <c r="H21" t="s">
+      <c r="I21" t="s">
+        <v>222</v>
+      </c>
+      <c r="J21" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80470_gloucestershire", ".\export_data\inspection_reports\80470_gloucestershire")</f>
+        <v>0</v>
+      </c>
+      <c r="K21" t="s">
         <v>223</v>
       </c>
-      <c r="I21" t="s">
-        <v>223</v>
-      </c>
-      <c r="J21" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80471_halton", ".\export_data\inspection_reports\80471_halton")</f>
-        <v>0</v>
-      </c>
-      <c r="K21" t="s">
+      <c r="L21" t="s">
+        <v>9</v>
+      </c>
+      <c r="M21" t="s">
+        <v>9</v>
+      </c>
+      <c r="N21" t="s">
         <v>224</v>
       </c>
-      <c r="L21" t="s">
-        <v>9</v>
-      </c>
-      <c r="M21" t="s">
+      <c r="O21" t="s">
         <v>225</v>
       </c>
-      <c r="N21" t="s">
+      <c r="P21" t="s">
         <v>226</v>
       </c>
-      <c r="O21" t="s">
-        <v>9</v>
-      </c>
-      <c r="P21" t="s">
-        <v>9</v>
-      </c>
       <c r="Q21" t="s">
-        <v>82</v>
+        <v>12</v>
       </c>
       <c r="R21" t="s">
-        <v>227</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22" spans="1:18">
       <c r="A22" t="s">
+        <v>227</v>
+      </c>
+      <c r="B22" t="s">
         <v>228</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
+        <v>27</v>
+      </c>
+      <c r="D22" t="s">
         <v>229</v>
       </c>
-      <c r="C22" t="s">
-        <v>50</v>
-      </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>230</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>231</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="G22" s="2" t="s">
+      <c r="H22" t="s">
         <v>233</v>
       </c>
-      <c r="H22" t="s">
+      <c r="I22" t="s">
+        <v>233</v>
+      </c>
+      <c r="J22" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80471_halton", ".\export_data\inspection_reports\80471_halton")</f>
+        <v>0</v>
+      </c>
+      <c r="K22" t="s">
         <v>234</v>
       </c>
-      <c r="I22" t="s">
+      <c r="L22" t="s">
+        <v>9</v>
+      </c>
+      <c r="M22" t="s">
         <v>235</v>
       </c>
-      <c r="J22" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80472_hampshire", ".\export_data\inspection_reports\80472_hampshire")</f>
-        <v>0</v>
-      </c>
-      <c r="K22" t="s">
+      <c r="N22" t="s">
         <v>236</v>
-      </c>
-      <c r="L22" t="s">
-        <v>9</v>
-      </c>
-      <c r="M22" t="s">
-        <v>237</v>
-      </c>
-      <c r="N22" t="s">
-        <v>238</v>
       </c>
       <c r="O22" t="s">
         <v>9</v>
@@ -3303,109 +3333,109 @@
         <v>82</v>
       </c>
       <c r="R22" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="23" spans="1:18">
       <c r="A23" t="s">
+        <v>238</v>
+      </c>
+      <c r="B23" t="s">
+        <v>239</v>
+      </c>
+      <c r="C23" t="s">
+        <v>50</v>
+      </c>
+      <c r="D23" t="s">
         <v>240</v>
       </c>
-      <c r="B23" t="s">
+      <c r="E23" t="s">
         <v>241</v>
       </c>
-      <c r="C23" t="s">
-        <v>15</v>
-      </c>
-      <c r="D23" t="s">
+      <c r="F23" t="s">
         <v>242</v>
       </c>
-      <c r="E23" t="s">
+      <c r="G23" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="F23" t="s">
+      <c r="H23" t="s">
         <v>244</v>
       </c>
-      <c r="G23" s="2" t="s">
+      <c r="I23" t="s">
         <v>245</v>
       </c>
-      <c r="H23" t="s">
+      <c r="J23" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80472_hampshire", ".\export_data\inspection_reports\80472_hampshire")</f>
+        <v>0</v>
+      </c>
+      <c r="K23" t="s">
         <v>246</v>
       </c>
-      <c r="I23" t="s">
-        <v>246</v>
-      </c>
-      <c r="J23" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80475_hertfordshire", ".\export_data\inspection_reports\80475_hertfordshire")</f>
-        <v>0</v>
-      </c>
-      <c r="K23" t="s">
+      <c r="L23" t="s">
+        <v>9</v>
+      </c>
+      <c r="M23" t="s">
         <v>247</v>
       </c>
-      <c r="L23" t="s">
-        <v>9</v>
-      </c>
-      <c r="M23" t="s">
+      <c r="N23" t="s">
         <v>248</v>
       </c>
-      <c r="N23" t="s">
+      <c r="O23" t="s">
+        <v>9</v>
+      </c>
+      <c r="P23" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>82</v>
+      </c>
+      <c r="R23" t="s">
         <v>249</v>
-      </c>
-      <c r="O23" t="s">
-        <v>250</v>
-      </c>
-      <c r="P23" t="s">
-        <v>251</v>
-      </c>
-      <c r="Q23" t="s">
-        <v>12</v>
-      </c>
-      <c r="R23" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="24" spans="1:18">
       <c r="A24" t="s">
+        <v>250</v>
+      </c>
+      <c r="B24" t="s">
+        <v>251</v>
+      </c>
+      <c r="C24" t="s">
+        <v>15</v>
+      </c>
+      <c r="D24" t="s">
         <v>252</v>
       </c>
-      <c r="B24" t="s">
+      <c r="E24" t="s">
         <v>253</v>
       </c>
-      <c r="C24" t="s">
-        <v>2</v>
-      </c>
-      <c r="D24" t="s">
+      <c r="F24" t="s">
         <v>254</v>
       </c>
-      <c r="E24" t="s">
+      <c r="G24" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="F24" t="s">
+      <c r="H24" t="s">
         <v>256</v>
       </c>
-      <c r="G24" s="2" t="s">
+      <c r="I24" t="s">
+        <v>256</v>
+      </c>
+      <c r="J24" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80475_hertfordshire", ".\export_data\inspection_reports\80475_hertfordshire")</f>
+        <v>0</v>
+      </c>
+      <c r="K24" t="s">
         <v>257</v>
       </c>
-      <c r="H24" t="s">
+      <c r="L24" t="s">
+        <v>9</v>
+      </c>
+      <c r="M24" t="s">
         <v>258</v>
       </c>
-      <c r="I24" t="s">
-        <v>258</v>
-      </c>
-      <c r="J24" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80478_kirklees", ".\export_data\inspection_reports\80478_kirklees")</f>
-        <v>0</v>
-      </c>
-      <c r="K24" t="s">
+      <c r="N24" t="s">
         <v>259</v>
-      </c>
-      <c r="L24" t="s">
-        <v>9</v>
-      </c>
-      <c r="M24" t="s">
-        <v>9</v>
-      </c>
-      <c r="N24" t="s">
-        <v>9</v>
       </c>
       <c r="O24" t="s">
         <v>260</v>
@@ -3428,7 +3458,7 @@
         <v>263</v>
       </c>
       <c r="C25" t="s">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="D25" t="s">
         <v>264</v>
@@ -3449,7 +3479,7 @@
         <v>268</v>
       </c>
       <c r="J25" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80480_lancashire", ".\export_data\inspection_reports\80480_lancashire")</f>
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80478_kirklees", ".\export_data\inspection_reports\80478_kirklees")</f>
         <v>0</v>
       </c>
       <c r="K25" t="s">
@@ -3462,13 +3492,13 @@
         <v>9</v>
       </c>
       <c r="N25" t="s">
+        <v>9</v>
+      </c>
+      <c r="O25" t="s">
         <v>270</v>
       </c>
-      <c r="O25" t="s">
+      <c r="P25" t="s">
         <v>271</v>
-      </c>
-      <c r="P25" t="s">
-        <v>272</v>
       </c>
       <c r="Q25" t="s">
         <v>12</v>
@@ -3479,34 +3509,34 @@
     </row>
     <row r="26" spans="1:18">
       <c r="A26" t="s">
+        <v>272</v>
+      </c>
+      <c r="B26" t="s">
         <v>273</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
+        <v>27</v>
+      </c>
+      <c r="D26" t="s">
         <v>274</v>
       </c>
-      <c r="C26" t="s">
-        <v>2</v>
-      </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>275</v>
       </c>
-      <c r="E26" t="s">
+      <c r="F26" t="s">
         <v>276</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G26" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="G26" s="2" t="s">
+      <c r="H26" t="s">
         <v>278</v>
       </c>
-      <c r="H26" t="s">
-        <v>268</v>
-      </c>
       <c r="I26" t="s">
-        <v>268</v>
+        <v>278</v>
       </c>
       <c r="J26" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80481_leeds", ".\export_data\inspection_reports\80481_leeds")</f>
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80480_lancashire", ".\export_data\inspection_reports\80480_lancashire")</f>
         <v>0</v>
       </c>
       <c r="K26" t="s">
@@ -3542,7 +3572,7 @@
         <v>284</v>
       </c>
       <c r="C27" t="s">
-        <v>174</v>
+        <v>2</v>
       </c>
       <c r="D27" t="s">
         <v>285</v>
@@ -3557,26 +3587,26 @@
         <v>288</v>
       </c>
       <c r="H27" t="s">
+        <v>278</v>
+      </c>
+      <c r="I27" t="s">
+        <v>278</v>
+      </c>
+      <c r="J27" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80481_leeds", ".\export_data\inspection_reports\80481_leeds")</f>
+        <v>0</v>
+      </c>
+      <c r="K27" t="s">
         <v>289</v>
       </c>
-      <c r="I27" t="s">
-        <v>289</v>
-      </c>
-      <c r="J27" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80483_leicestershire", ".\export_data\inspection_reports\80483_leicestershire")</f>
-        <v>0</v>
-      </c>
-      <c r="K27" t="s">
+      <c r="L27" t="s">
+        <v>9</v>
+      </c>
+      <c r="M27" t="s">
+        <v>9</v>
+      </c>
+      <c r="N27" t="s">
         <v>290</v>
-      </c>
-      <c r="L27" t="s">
-        <v>9</v>
-      </c>
-      <c r="M27" t="s">
-        <v>9</v>
-      </c>
-      <c r="N27" t="s">
-        <v>68</v>
       </c>
       <c r="O27" t="s">
         <v>291</v>
@@ -3617,308 +3647,308 @@
         <v>299</v>
       </c>
       <c r="I28" t="s">
+        <v>299</v>
+      </c>
+      <c r="J28" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80483_leicestershire", ".\export_data\inspection_reports\80483_leicestershire")</f>
+        <v>0</v>
+      </c>
+      <c r="K28" t="s">
         <v>300</v>
       </c>
-      <c r="J28" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80484_lincolnshire", ".\export_data\inspection_reports\80484_lincolnshire")</f>
-        <v>0</v>
-      </c>
-      <c r="K28" t="s">
+      <c r="L28" t="s">
+        <v>9</v>
+      </c>
+      <c r="M28" t="s">
+        <v>9</v>
+      </c>
+      <c r="N28" t="s">
+        <v>68</v>
+      </c>
+      <c r="O28" t="s">
         <v>301</v>
       </c>
-      <c r="L28" t="s">
-        <v>9</v>
-      </c>
-      <c r="M28" t="s">
+      <c r="P28" t="s">
         <v>302</v>
       </c>
-      <c r="N28" t="s">
-        <v>303</v>
-      </c>
-      <c r="O28" t="s">
-        <v>9</v>
-      </c>
-      <c r="P28" t="s">
-        <v>9</v>
-      </c>
       <c r="Q28" t="s">
-        <v>82</v>
+        <v>12</v>
       </c>
       <c r="R28" t="s">
-        <v>304</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29" spans="1:18">
       <c r="A29" t="s">
+        <v>303</v>
+      </c>
+      <c r="B29" t="s">
+        <v>304</v>
+      </c>
+      <c r="C29" t="s">
+        <v>174</v>
+      </c>
+      <c r="D29" t="s">
         <v>305</v>
       </c>
-      <c r="B29" t="s">
+      <c r="E29" t="s">
         <v>306</v>
       </c>
-      <c r="C29" t="s">
-        <v>27</v>
-      </c>
-      <c r="D29" t="s">
+      <c r="F29" t="s">
         <v>307</v>
       </c>
-      <c r="E29" t="s">
+      <c r="G29" s="2" t="s">
         <v>308</v>
       </c>
-      <c r="F29" t="s">
+      <c r="H29" t="s">
         <v>309</v>
       </c>
-      <c r="G29" s="2" t="s">
+      <c r="I29" t="s">
         <v>310</v>
       </c>
-      <c r="H29" t="s">
+      <c r="J29" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80484_lincolnshire", ".\export_data\inspection_reports\80484_lincolnshire")</f>
+        <v>0</v>
+      </c>
+      <c r="K29" t="s">
         <v>311</v>
       </c>
-      <c r="I29" t="s">
+      <c r="L29" t="s">
+        <v>9</v>
+      </c>
+      <c r="M29" t="s">
         <v>312</v>
       </c>
-      <c r="J29" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80485_liverpool", ".\export_data\inspection_reports\80485_liverpool")</f>
-        <v>0</v>
-      </c>
-      <c r="K29" t="s">
+      <c r="N29" t="s">
         <v>313</v>
       </c>
-      <c r="L29" t="s">
+      <c r="O29" t="s">
+        <v>9</v>
+      </c>
+      <c r="P29" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>82</v>
+      </c>
+      <c r="R29" t="s">
         <v>314</v>
-      </c>
-      <c r="M29" t="s">
-        <v>315</v>
-      </c>
-      <c r="N29" t="s">
-        <v>316</v>
-      </c>
-      <c r="O29" t="s">
-        <v>9</v>
-      </c>
-      <c r="P29" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q29" t="s">
-        <v>317</v>
-      </c>
-      <c r="R29" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="30" spans="1:18">
       <c r="A30" t="s">
+        <v>315</v>
+      </c>
+      <c r="B30" t="s">
+        <v>316</v>
+      </c>
+      <c r="C30" t="s">
+        <v>27</v>
+      </c>
+      <c r="D30" t="s">
+        <v>317</v>
+      </c>
+      <c r="E30" t="s">
+        <v>318</v>
+      </c>
+      <c r="F30" t="s">
         <v>319</v>
       </c>
-      <c r="B30" t="s">
+      <c r="G30" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="C30" t="s">
+      <c r="H30" t="s">
         <v>321</v>
       </c>
-      <c r="D30" t="s">
+      <c r="I30" t="s">
         <v>322</v>
       </c>
-      <c r="E30" t="s">
+      <c r="J30" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80485_liverpool", ".\export_data\inspection_reports\80485_liverpool")</f>
+        <v>0</v>
+      </c>
+      <c r="K30" t="s">
         <v>323</v>
       </c>
-      <c r="F30" t="s">
+      <c r="L30" t="s">
         <v>324</v>
       </c>
-      <c r="G30" s="2" t="s">
+      <c r="M30" t="s">
         <v>325</v>
       </c>
-      <c r="H30" t="s">
+      <c r="N30" t="s">
         <v>326</v>
       </c>
-      <c r="I30" t="s">
-        <v>326</v>
-      </c>
-      <c r="J30" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80488_bexley", ".\export_data\inspection_reports\80488_bexley")</f>
-        <v>0</v>
-      </c>
-      <c r="K30" t="s">
+      <c r="O30" t="s">
+        <v>9</v>
+      </c>
+      <c r="P30" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q30" t="s">
         <v>327</v>
       </c>
-      <c r="L30" t="s">
-        <v>9</v>
-      </c>
-      <c r="M30" t="s">
+      <c r="R30" t="s">
         <v>328</v>
-      </c>
-      <c r="N30" t="s">
-        <v>329</v>
-      </c>
-      <c r="O30" t="s">
-        <v>9</v>
-      </c>
-      <c r="P30" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q30" t="s">
-        <v>82</v>
-      </c>
-      <c r="R30" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="31" spans="1:18">
       <c r="A31" t="s">
+        <v>329</v>
+      </c>
+      <c r="B31" t="s">
+        <v>330</v>
+      </c>
+      <c r="C31" t="s">
         <v>331</v>
       </c>
-      <c r="B31" t="s">
+      <c r="D31" t="s">
         <v>332</v>
       </c>
-      <c r="C31" t="s">
-        <v>321</v>
-      </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>333</v>
       </c>
-      <c r="E31" t="s">
+      <c r="F31" t="s">
         <v>334</v>
       </c>
-      <c r="F31" t="s">
+      <c r="G31" s="2" t="s">
         <v>335</v>
       </c>
-      <c r="G31" s="2" t="s">
+      <c r="H31" t="s">
         <v>336</v>
       </c>
-      <c r="H31" t="s">
+      <c r="I31" t="s">
+        <v>336</v>
+      </c>
+      <c r="J31" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80488_bexley", ".\export_data\inspection_reports\80488_bexley")</f>
+        <v>0</v>
+      </c>
+      <c r="K31" t="s">
         <v>337</v>
       </c>
-      <c r="I31" t="s">
-        <v>337</v>
-      </c>
-      <c r="J31" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80490_bromley", ".\export_data\inspection_reports\80490_bromley")</f>
-        <v>0</v>
-      </c>
-      <c r="K31" t="s">
+      <c r="L31" t="s">
+        <v>9</v>
+      </c>
+      <c r="M31" t="s">
         <v>338</v>
-      </c>
-      <c r="L31" t="s">
-        <v>9</v>
-      </c>
-      <c r="M31" t="s">
-        <v>9</v>
       </c>
       <c r="N31" t="s">
         <v>339</v>
       </c>
       <c r="O31" t="s">
+        <v>9</v>
+      </c>
+      <c r="P31" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>82</v>
+      </c>
+      <c r="R31" t="s">
         <v>340</v>
-      </c>
-      <c r="P31" t="s">
-        <v>341</v>
-      </c>
-      <c r="Q31" t="s">
-        <v>12</v>
-      </c>
-      <c r="R31" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="32" spans="1:18">
       <c r="A32" t="s">
+        <v>341</v>
+      </c>
+      <c r="B32" t="s">
         <v>342</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C32" t="s">
+        <v>331</v>
+      </c>
+      <c r="D32" t="s">
         <v>343</v>
       </c>
-      <c r="C32" t="s">
-        <v>321</v>
-      </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
         <v>344</v>
       </c>
-      <c r="E32" t="s">
+      <c r="F32" t="s">
         <v>345</v>
       </c>
-      <c r="F32" t="s">
+      <c r="G32" s="2" t="s">
         <v>346</v>
       </c>
-      <c r="G32" s="2" t="s">
+      <c r="H32" t="s">
         <v>347</v>
       </c>
-      <c r="H32" t="s">
+      <c r="I32" t="s">
+        <v>347</v>
+      </c>
+      <c r="J32" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80490_bromley", ".\export_data\inspection_reports\80490_bromley")</f>
+        <v>0</v>
+      </c>
+      <c r="K32" t="s">
         <v>348</v>
       </c>
-      <c r="I32" t="s">
-        <v>348</v>
-      </c>
-      <c r="J32" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80492_croydon", ".\export_data\inspection_reports\80492_croydon")</f>
-        <v>0</v>
-      </c>
-      <c r="K32" t="s">
+      <c r="L32" t="s">
+        <v>9</v>
+      </c>
+      <c r="M32" t="s">
+        <v>9</v>
+      </c>
+      <c r="N32" t="s">
         <v>349</v>
       </c>
-      <c r="L32" t="s">
-        <v>9</v>
-      </c>
-      <c r="M32" t="s">
+      <c r="O32" t="s">
         <v>350</v>
       </c>
-      <c r="N32" t="s">
+      <c r="P32" t="s">
         <v>351</v>
       </c>
-      <c r="O32" t="s">
-        <v>9</v>
-      </c>
-      <c r="P32" t="s">
-        <v>9</v>
-      </c>
       <c r="Q32" t="s">
-        <v>82</v>
+        <v>12</v>
       </c>
       <c r="R32" t="s">
-        <v>352</v>
+        <v>9</v>
       </c>
     </row>
     <row r="33" spans="1:18">
       <c r="A33" t="s">
+        <v>352</v>
+      </c>
+      <c r="B33" t="s">
         <v>353</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
+        <v>331</v>
+      </c>
+      <c r="D33" t="s">
         <v>354</v>
       </c>
-      <c r="C33" t="s">
-        <v>321</v>
-      </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
         <v>355</v>
       </c>
-      <c r="E33" t="s">
+      <c r="F33" t="s">
         <v>356</v>
       </c>
-      <c r="F33" t="s">
+      <c r="G33" s="2" t="s">
         <v>357</v>
       </c>
-      <c r="G33" s="2" t="s">
+      <c r="H33" t="s">
         <v>358</v>
       </c>
-      <c r="H33" t="s">
+      <c r="I33" t="s">
+        <v>358</v>
+      </c>
+      <c r="J33" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80492_croydon", ".\export_data\inspection_reports\80492_croydon")</f>
+        <v>0</v>
+      </c>
+      <c r="K33" t="s">
         <v>359</v>
       </c>
-      <c r="I33" t="s">
-        <v>359</v>
-      </c>
-      <c r="J33" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80495_greenwich", ".\export_data\inspection_reports\80495_greenwich")</f>
-        <v>0</v>
-      </c>
-      <c r="K33" t="s">
+      <c r="L33" t="s">
+        <v>9</v>
+      </c>
+      <c r="M33" t="s">
         <v>360</v>
       </c>
-      <c r="L33" t="s">
-        <v>9</v>
-      </c>
-      <c r="M33" t="s">
+      <c r="N33" t="s">
         <v>361</v>
-      </c>
-      <c r="N33" t="s">
-        <v>362</v>
       </c>
       <c r="O33" t="s">
         <v>9</v>
@@ -3930,52 +3960,52 @@
         <v>82</v>
       </c>
       <c r="R33" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="34" spans="1:18">
       <c r="A34" t="s">
+        <v>363</v>
+      </c>
+      <c r="B34" t="s">
         <v>364</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
+        <v>331</v>
+      </c>
+      <c r="D34" t="s">
         <v>365</v>
       </c>
-      <c r="C34" t="s">
-        <v>321</v>
-      </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
         <v>366</v>
       </c>
-      <c r="E34" t="s">
+      <c r="F34" t="s">
         <v>367</v>
       </c>
-      <c r="F34" t="s">
+      <c r="G34" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="G34" s="2" t="s">
+      <c r="H34" t="s">
         <v>369</v>
       </c>
-      <c r="H34" t="s">
+      <c r="I34" t="s">
+        <v>369</v>
+      </c>
+      <c r="J34" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80495_greenwich", ".\export_data\inspection_reports\80495_greenwich")</f>
+        <v>0</v>
+      </c>
+      <c r="K34" t="s">
         <v>370</v>
       </c>
-      <c r="I34" t="s">
-        <v>370</v>
-      </c>
-      <c r="J34" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80498_haringey", ".\export_data\inspection_reports\80498_haringey")</f>
-        <v>0</v>
-      </c>
-      <c r="K34" t="s">
+      <c r="L34" t="s">
+        <v>9</v>
+      </c>
+      <c r="M34" t="s">
         <v>371</v>
       </c>
-      <c r="L34" t="s">
-        <v>9</v>
-      </c>
-      <c r="M34" t="s">
+      <c r="N34" t="s">
         <v>372</v>
-      </c>
-      <c r="N34" t="s">
-        <v>373</v>
       </c>
       <c r="O34" t="s">
         <v>9</v>
@@ -3987,115 +4017,115 @@
         <v>82</v>
       </c>
       <c r="R34" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="35" spans="1:18">
       <c r="A35" t="s">
+        <v>374</v>
+      </c>
+      <c r="B35" t="s">
         <v>375</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
+        <v>331</v>
+      </c>
+      <c r="D35" t="s">
         <v>376</v>
       </c>
-      <c r="C35" t="s">
-        <v>321</v>
-      </c>
-      <c r="D35" t="s">
+      <c r="E35" t="s">
         <v>377</v>
       </c>
-      <c r="E35" t="s">
+      <c r="F35" t="s">
         <v>378</v>
       </c>
-      <c r="F35" t="s">
+      <c r="G35" s="2" t="s">
         <v>379</v>
       </c>
-      <c r="G35" s="2" t="s">
+      <c r="H35" t="s">
         <v>380</v>
       </c>
-      <c r="H35" t="s">
+      <c r="I35" t="s">
+        <v>380</v>
+      </c>
+      <c r="J35" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80498_haringey", ".\export_data\inspection_reports\80498_haringey")</f>
+        <v>0</v>
+      </c>
+      <c r="K35" t="s">
         <v>381</v>
       </c>
-      <c r="I35" t="s">
-        <v>381</v>
-      </c>
-      <c r="J35" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80499_harrow", ".\export_data\inspection_reports\80499_harrow")</f>
-        <v>0</v>
-      </c>
-      <c r="K35" t="s">
+      <c r="L35" t="s">
+        <v>9</v>
+      </c>
+      <c r="M35" t="s">
         <v>382</v>
-      </c>
-      <c r="L35" t="s">
-        <v>9</v>
-      </c>
-      <c r="M35" t="s">
-        <v>9</v>
       </c>
       <c r="N35" t="s">
         <v>383</v>
       </c>
       <c r="O35" t="s">
+        <v>9</v>
+      </c>
+      <c r="P35" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>82</v>
+      </c>
+      <c r="R35" t="s">
         <v>384</v>
-      </c>
-      <c r="P35" t="s">
-        <v>385</v>
-      </c>
-      <c r="Q35" t="s">
-        <v>12</v>
-      </c>
-      <c r="R35" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="36" spans="1:18">
       <c r="A36" t="s">
+        <v>385</v>
+      </c>
+      <c r="B36" t="s">
         <v>386</v>
       </c>
-      <c r="B36" t="s">
+      <c r="C36" t="s">
+        <v>331</v>
+      </c>
+      <c r="D36" t="s">
         <v>387</v>
       </c>
-      <c r="C36" t="s">
-        <v>321</v>
-      </c>
-      <c r="D36" t="s">
+      <c r="E36" t="s">
         <v>388</v>
       </c>
-      <c r="E36" t="s">
+      <c r="F36" t="s">
         <v>389</v>
       </c>
-      <c r="F36" t="s">
+      <c r="G36" s="2" t="s">
         <v>390</v>
       </c>
-      <c r="G36" s="2" t="s">
+      <c r="H36" t="s">
         <v>391</v>
       </c>
-      <c r="H36" t="s">
+      <c r="I36" t="s">
+        <v>391</v>
+      </c>
+      <c r="J36" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80499_harrow", ".\export_data\inspection_reports\80499_harrow")</f>
+        <v>0</v>
+      </c>
+      <c r="K36" t="s">
         <v>392</v>
       </c>
-      <c r="I36" t="s">
-        <v>392</v>
-      </c>
-      <c r="J36" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80501_hillingdon", ".\export_data\inspection_reports\80501_hillingdon")</f>
-        <v>0</v>
-      </c>
-      <c r="K36" t="s">
+      <c r="L36" t="s">
+        <v>9</v>
+      </c>
+      <c r="M36" t="s">
+        <v>9</v>
+      </c>
+      <c r="N36" t="s">
         <v>393</v>
       </c>
-      <c r="L36" t="s">
-        <v>9</v>
-      </c>
-      <c r="M36" t="s">
-        <v>9</v>
-      </c>
-      <c r="N36" t="s">
+      <c r="O36" t="s">
         <v>394</v>
       </c>
-      <c r="O36" t="s">
+      <c r="P36" t="s">
         <v>395</v>
-      </c>
-      <c r="P36" t="s">
-        <v>396</v>
       </c>
       <c r="Q36" t="s">
         <v>12</v>
@@ -4106,116 +4136,116 @@
     </row>
     <row r="37" spans="1:18">
       <c r="A37" t="s">
+        <v>396</v>
+      </c>
+      <c r="B37" t="s">
         <v>397</v>
       </c>
-      <c r="B37" t="s">
+      <c r="C37" t="s">
+        <v>331</v>
+      </c>
+      <c r="D37" t="s">
         <v>398</v>
       </c>
-      <c r="C37" t="s">
-        <v>321</v>
-      </c>
-      <c r="D37" t="s">
+      <c r="E37" t="s">
         <v>399</v>
       </c>
-      <c r="E37" t="s">
+      <c r="F37" t="s">
         <v>400</v>
       </c>
-      <c r="F37" t="s">
+      <c r="G37" s="2" t="s">
         <v>401</v>
       </c>
-      <c r="G37" s="2" t="s">
+      <c r="H37" t="s">
         <v>402</v>
       </c>
-      <c r="H37" t="s">
+      <c r="I37" t="s">
+        <v>402</v>
+      </c>
+      <c r="J37" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80501_hillingdon", ".\export_data\inspection_reports\80501_hillingdon")</f>
+        <v>0</v>
+      </c>
+      <c r="K37" t="s">
         <v>403</v>
       </c>
-      <c r="I37" t="s">
-        <v>403</v>
-      </c>
-      <c r="J37" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80503_hounslow", ".\export_data\inspection_reports\80503_hounslow")</f>
-        <v>0</v>
-      </c>
-      <c r="K37" t="s">
+      <c r="L37" t="s">
+        <v>9</v>
+      </c>
+      <c r="M37" t="s">
+        <v>9</v>
+      </c>
+      <c r="N37" t="s">
         <v>404</v>
       </c>
-      <c r="L37" t="s">
-        <v>9</v>
-      </c>
-      <c r="M37" t="s">
+      <c r="O37" t="s">
         <v>405</v>
       </c>
-      <c r="N37" t="s">
+      <c r="P37" t="s">
         <v>406</v>
       </c>
-      <c r="O37" t="s">
-        <v>9</v>
-      </c>
-      <c r="P37" t="s">
-        <v>9</v>
-      </c>
       <c r="Q37" t="s">
-        <v>82</v>
+        <v>12</v>
       </c>
       <c r="R37" t="s">
-        <v>407</v>
+        <v>9</v>
       </c>
     </row>
     <row r="38" spans="1:18">
       <c r="A38" t="s">
+        <v>407</v>
+      </c>
+      <c r="B38" t="s">
         <v>408</v>
       </c>
-      <c r="B38" t="s">
+      <c r="C38" t="s">
+        <v>331</v>
+      </c>
+      <c r="D38" t="s">
         <v>409</v>
       </c>
-      <c r="C38" t="s">
-        <v>321</v>
-      </c>
-      <c r="D38" t="s">
+      <c r="E38" t="s">
         <v>410</v>
       </c>
-      <c r="E38" t="s">
+      <c r="F38" t="s">
         <v>411</v>
       </c>
-      <c r="F38" t="s">
+      <c r="G38" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="G38" s="2" t="s">
+      <c r="H38" t="s">
         <v>413</v>
       </c>
-      <c r="H38" t="s">
+      <c r="I38" t="s">
+        <v>413</v>
+      </c>
+      <c r="J38" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80503_hounslow", ".\export_data\inspection_reports\80503_hounslow")</f>
+        <v>0</v>
+      </c>
+      <c r="K38" t="s">
         <v>414</v>
       </c>
-      <c r="I38" t="s">
-        <v>414</v>
-      </c>
-      <c r="J38" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80505_islington", ".\export_data\inspection_reports\80505_islington")</f>
-        <v>0</v>
-      </c>
-      <c r="K38" t="s">
+      <c r="L38" t="s">
+        <v>9</v>
+      </c>
+      <c r="M38" t="s">
         <v>415</v>
       </c>
-      <c r="L38" t="s">
-        <v>9</v>
-      </c>
-      <c r="M38" t="s">
+      <c r="N38" t="s">
         <v>416</v>
       </c>
-      <c r="N38" t="s">
+      <c r="O38" t="s">
+        <v>9</v>
+      </c>
+      <c r="P38" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>82</v>
+      </c>
+      <c r="R38" t="s">
         <v>417</v>
-      </c>
-      <c r="O38" t="s">
-        <v>9</v>
-      </c>
-      <c r="P38" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q38" t="s">
-        <v>12</v>
-      </c>
-      <c r="R38" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="39" spans="1:18">
@@ -4226,7 +4256,7 @@
         <v>419</v>
       </c>
       <c r="C39" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
       <c r="D39" t="s">
         <v>420</v>
@@ -4247,7 +4277,7 @@
         <v>424</v>
       </c>
       <c r="J39" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80508_lewisham", ".\export_data\inspection_reports\80508_lewisham")</f>
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80505_islington", ".\export_data\inspection_reports\80505_islington")</f>
         <v>0</v>
       </c>
       <c r="K39" t="s">
@@ -4257,16 +4287,16 @@
         <v>9</v>
       </c>
       <c r="M39" t="s">
-        <v>9</v>
+        <v>426</v>
       </c>
       <c r="N39" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="O39" t="s">
-        <v>427</v>
+        <v>9</v>
       </c>
       <c r="P39" t="s">
-        <v>428</v>
+        <v>9</v>
       </c>
       <c r="Q39" t="s">
         <v>12</v>
@@ -4277,53 +4307,53 @@
     </row>
     <row r="40" spans="1:18">
       <c r="A40" t="s">
+        <v>428</v>
+      </c>
+      <c r="B40" t="s">
         <v>429</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" t="s">
+        <v>331</v>
+      </c>
+      <c r="D40" t="s">
         <v>430</v>
       </c>
-      <c r="C40" t="s">
-        <v>321</v>
-      </c>
-      <c r="D40" t="s">
+      <c r="E40" t="s">
         <v>431</v>
       </c>
-      <c r="E40" t="s">
+      <c r="F40" t="s">
         <v>432</v>
       </c>
-      <c r="F40" t="s">
+      <c r="G40" s="2" t="s">
         <v>433</v>
       </c>
-      <c r="G40" s="2" t="s">
+      <c r="H40" t="s">
         <v>434</v>
       </c>
-      <c r="H40" t="s">
+      <c r="I40" t="s">
+        <v>434</v>
+      </c>
+      <c r="J40" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80508_lewisham", ".\export_data\inspection_reports\80508_lewisham")</f>
+        <v>0</v>
+      </c>
+      <c r="K40" t="s">
         <v>435</v>
       </c>
-      <c r="I40" t="s">
-        <v>435</v>
-      </c>
-      <c r="J40" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80510_merton", ".\export_data\inspection_reports\80510_merton")</f>
-        <v>0</v>
-      </c>
-      <c r="K40" t="s">
+      <c r="L40" t="s">
+        <v>9</v>
+      </c>
+      <c r="M40" t="s">
+        <v>9</v>
+      </c>
+      <c r="N40" t="s">
         <v>436</v>
       </c>
-      <c r="L40" t="s">
-        <v>9</v>
-      </c>
-      <c r="M40" t="s">
-        <v>9</v>
-      </c>
-      <c r="N40" t="s">
+      <c r="O40" t="s">
         <v>437</v>
       </c>
-      <c r="O40" t="s">
+      <c r="P40" t="s">
         <v>438</v>
-      </c>
-      <c r="P40" t="s">
-        <v>439</v>
       </c>
       <c r="Q40" t="s">
         <v>12</v>
@@ -4334,53 +4364,53 @@
     </row>
     <row r="41" spans="1:18">
       <c r="A41" t="s">
+        <v>439</v>
+      </c>
+      <c r="B41" t="s">
         <v>440</v>
       </c>
-      <c r="B41" t="s">
+      <c r="C41" t="s">
+        <v>331</v>
+      </c>
+      <c r="D41" t="s">
         <v>441</v>
       </c>
-      <c r="C41" t="s">
-        <v>321</v>
-      </c>
-      <c r="D41" t="s">
+      <c r="E41" t="s">
         <v>442</v>
       </c>
-      <c r="E41" t="s">
+      <c r="F41" t="s">
         <v>443</v>
       </c>
-      <c r="F41" t="s">
+      <c r="G41" s="2" t="s">
         <v>444</v>
       </c>
-      <c r="G41" s="2" t="s">
+      <c r="H41" t="s">
         <v>445</v>
       </c>
-      <c r="H41" t="s">
+      <c r="I41" t="s">
+        <v>445</v>
+      </c>
+      <c r="J41" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80510_merton", ".\export_data\inspection_reports\80510_merton")</f>
+        <v>0</v>
+      </c>
+      <c r="K41" t="s">
         <v>446</v>
       </c>
-      <c r="I41" t="s">
-        <v>446</v>
-      </c>
-      <c r="J41" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80513_richmond upon thames", ".\export_data\inspection_reports\80513_richmond upon thames")</f>
-        <v>0</v>
-      </c>
-      <c r="K41" t="s">
+      <c r="L41" t="s">
+        <v>9</v>
+      </c>
+      <c r="M41" t="s">
+        <v>9</v>
+      </c>
+      <c r="N41" t="s">
         <v>447</v>
       </c>
-      <c r="L41" t="s">
-        <v>9</v>
-      </c>
-      <c r="M41" t="s">
-        <v>9</v>
-      </c>
-      <c r="N41" t="s">
+      <c r="O41" t="s">
         <v>448</v>
       </c>
-      <c r="O41" t="s">
+      <c r="P41" t="s">
         <v>449</v>
-      </c>
-      <c r="P41" t="s">
-        <v>450</v>
       </c>
       <c r="Q41" t="s">
         <v>12</v>
@@ -4391,53 +4421,53 @@
     </row>
     <row r="42" spans="1:18">
       <c r="A42" t="s">
+        <v>450</v>
+      </c>
+      <c r="B42" t="s">
         <v>451</v>
       </c>
-      <c r="B42" t="s">
+      <c r="C42" t="s">
+        <v>331</v>
+      </c>
+      <c r="D42" t="s">
         <v>452</v>
       </c>
-      <c r="C42" t="s">
-        <v>321</v>
-      </c>
-      <c r="D42" t="s">
+      <c r="E42" t="s">
         <v>453</v>
       </c>
-      <c r="E42" t="s">
+      <c r="F42" t="s">
         <v>454</v>
       </c>
-      <c r="F42" t="s">
+      <c r="G42" s="2" t="s">
         <v>455</v>
       </c>
-      <c r="G42" s="2" t="s">
+      <c r="H42" t="s">
         <v>456</v>
       </c>
-      <c r="H42" t="s">
+      <c r="I42" t="s">
+        <v>456</v>
+      </c>
+      <c r="J42" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80513_richmond upon thames", ".\export_data\inspection_reports\80513_richmond upon thames")</f>
+        <v>0</v>
+      </c>
+      <c r="K42" t="s">
         <v>457</v>
       </c>
-      <c r="I42" t="s">
-        <v>457</v>
-      </c>
-      <c r="J42" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80515_sutton", ".\export_data\inspection_reports\80515_sutton")</f>
-        <v>0</v>
-      </c>
-      <c r="K42" t="s">
+      <c r="L42" t="s">
+        <v>9</v>
+      </c>
+      <c r="M42" t="s">
+        <v>9</v>
+      </c>
+      <c r="N42" t="s">
         <v>458</v>
       </c>
-      <c r="L42" t="s">
-        <v>9</v>
-      </c>
-      <c r="M42" t="s">
-        <v>9</v>
-      </c>
-      <c r="N42" t="s">
+      <c r="O42" t="s">
         <v>459</v>
       </c>
-      <c r="O42" t="s">
+      <c r="P42" t="s">
         <v>460</v>
-      </c>
-      <c r="P42" t="s">
-        <v>461</v>
       </c>
       <c r="Q42" t="s">
         <v>12</v>
@@ -4448,47 +4478,47 @@
     </row>
     <row r="43" spans="1:18">
       <c r="A43" t="s">
+        <v>461</v>
+      </c>
+      <c r="B43" t="s">
         <v>462</v>
       </c>
-      <c r="B43" t="s">
+      <c r="C43" t="s">
+        <v>331</v>
+      </c>
+      <c r="D43" t="s">
         <v>463</v>
       </c>
-      <c r="C43" t="s">
-        <v>321</v>
-      </c>
-      <c r="D43" t="s">
+      <c r="E43" t="s">
         <v>464</v>
       </c>
-      <c r="E43" t="s">
+      <c r="F43" t="s">
         <v>465</v>
       </c>
-      <c r="F43" t="s">
+      <c r="G43" s="2" t="s">
         <v>466</v>
       </c>
-      <c r="G43" s="2" t="s">
+      <c r="H43" t="s">
         <v>467</v>
       </c>
-      <c r="H43" t="s">
+      <c r="I43" t="s">
+        <v>467</v>
+      </c>
+      <c r="J43" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80515_sutton", ".\export_data\inspection_reports\80515_sutton")</f>
+        <v>0</v>
+      </c>
+      <c r="K43" t="s">
         <v>468</v>
       </c>
-      <c r="I43" t="s">
-        <v>468</v>
-      </c>
-      <c r="J43" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80516_tower hamlets", ".\export_data\inspection_reports\80516_tower hamlets")</f>
-        <v>0</v>
-      </c>
-      <c r="K43" t="s">
+      <c r="L43" t="s">
+        <v>9</v>
+      </c>
+      <c r="M43" t="s">
+        <v>9</v>
+      </c>
+      <c r="N43" t="s">
         <v>469</v>
-      </c>
-      <c r="L43" t="s">
-        <v>9</v>
-      </c>
-      <c r="M43" t="s">
-        <v>9</v>
-      </c>
-      <c r="N43" t="s">
-        <v>68</v>
       </c>
       <c r="O43" t="s">
         <v>470</v>
@@ -4511,7 +4541,7 @@
         <v>473</v>
       </c>
       <c r="C44" t="s">
-        <v>27</v>
+        <v>331</v>
       </c>
       <c r="D44" t="s">
         <v>474</v>
@@ -4532,7 +4562,7 @@
         <v>478</v>
       </c>
       <c r="J44" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80521_manchester", ".\export_data\inspection_reports\80521_manchester")</f>
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80516_tower hamlets", ".\export_data\inspection_reports\80516_tower hamlets")</f>
         <v>0</v>
       </c>
       <c r="K44" t="s">
@@ -4545,13 +4575,13 @@
         <v>9</v>
       </c>
       <c r="N44" t="s">
+        <v>68</v>
+      </c>
+      <c r="O44" t="s">
         <v>480</v>
       </c>
-      <c r="O44" t="s">
+      <c r="P44" t="s">
         <v>481</v>
-      </c>
-      <c r="P44" t="s">
-        <v>482</v>
       </c>
       <c r="Q44" t="s">
         <v>12</v>
@@ -4562,224 +4592,224 @@
     </row>
     <row r="45" spans="1:18">
       <c r="A45" t="s">
+        <v>482</v>
+      </c>
+      <c r="B45" t="s">
         <v>483</v>
       </c>
-      <c r="B45" t="s">
+      <c r="C45" t="s">
+        <v>27</v>
+      </c>
+      <c r="D45" t="s">
         <v>484</v>
       </c>
-      <c r="C45" t="s">
+      <c r="E45" t="s">
         <v>485</v>
       </c>
-      <c r="D45" t="s">
+      <c r="F45" t="s">
         <v>486</v>
       </c>
-      <c r="E45" t="s">
+      <c r="G45" s="2" t="s">
         <v>487</v>
       </c>
-      <c r="F45" t="s">
+      <c r="H45" t="s">
         <v>488</v>
       </c>
-      <c r="G45" s="2" t="s">
+      <c r="I45" t="s">
+        <v>488</v>
+      </c>
+      <c r="J45" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80521_manchester", ".\export_data\inspection_reports\80521_manchester")</f>
+        <v>0</v>
+      </c>
+      <c r="K45" t="s">
         <v>489</v>
       </c>
-      <c r="H45" t="s">
+      <c r="L45" t="s">
+        <v>9</v>
+      </c>
+      <c r="M45" t="s">
+        <v>9</v>
+      </c>
+      <c r="N45" t="s">
         <v>490</v>
       </c>
-      <c r="I45" t="s">
-        <v>490</v>
-      </c>
-      <c r="J45" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80522_medway", ".\export_data\inspection_reports\80522_medway")</f>
-        <v>0</v>
-      </c>
-      <c r="K45" t="s">
+      <c r="O45" t="s">
         <v>491</v>
       </c>
-      <c r="L45" t="s">
-        <v>9</v>
-      </c>
-      <c r="M45" t="s">
+      <c r="P45" t="s">
         <v>492</v>
       </c>
-      <c r="N45" t="s">
-        <v>493</v>
-      </c>
-      <c r="O45" t="s">
-        <v>9</v>
-      </c>
-      <c r="P45" t="s">
-        <v>9</v>
-      </c>
       <c r="Q45" t="s">
-        <v>494</v>
+        <v>12</v>
       </c>
       <c r="R45" t="s">
-        <v>495</v>
+        <v>9</v>
       </c>
     </row>
     <row r="46" spans="1:18">
       <c r="A46" t="s">
+        <v>493</v>
+      </c>
+      <c r="B46" t="s">
+        <v>494</v>
+      </c>
+      <c r="C46" t="s">
+        <v>495</v>
+      </c>
+      <c r="D46" t="s">
         <v>496</v>
       </c>
-      <c r="B46" t="s">
+      <c r="E46" t="s">
         <v>497</v>
       </c>
-      <c r="C46" t="s">
-        <v>50</v>
-      </c>
-      <c r="D46" t="s">
+      <c r="F46" t="s">
         <v>498</v>
       </c>
-      <c r="E46" t="s">
+      <c r="G46" s="2" t="s">
         <v>499</v>
       </c>
-      <c r="F46" t="s">
+      <c r="H46" t="s">
         <v>500</v>
       </c>
-      <c r="G46" s="2" t="s">
+      <c r="I46" t="s">
+        <v>500</v>
+      </c>
+      <c r="J46" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80522_medway", ".\export_data\inspection_reports\80522_medway")</f>
+        <v>0</v>
+      </c>
+      <c r="K46" t="s">
         <v>501</v>
       </c>
-      <c r="H46" t="s">
+      <c r="L46" t="s">
+        <v>9</v>
+      </c>
+      <c r="M46" t="s">
         <v>502</v>
       </c>
-      <c r="I46" t="s">
-        <v>502</v>
-      </c>
-      <c r="J46" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80524_milton keynes", ".\export_data\inspection_reports\80524_milton keynes")</f>
-        <v>0</v>
-      </c>
-      <c r="K46" t="s">
+      <c r="N46" t="s">
         <v>503</v>
       </c>
-      <c r="L46" t="s">
-        <v>9</v>
-      </c>
-      <c r="M46" t="s">
+      <c r="O46" t="s">
+        <v>9</v>
+      </c>
+      <c r="P46" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q46" t="s">
         <v>504</v>
       </c>
-      <c r="N46" t="s">
+      <c r="R46" t="s">
         <v>505</v>
-      </c>
-      <c r="O46" t="s">
-        <v>9</v>
-      </c>
-      <c r="P46" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q46" t="s">
-        <v>82</v>
-      </c>
-      <c r="R46" t="s">
-        <v>506</v>
       </c>
     </row>
     <row r="47" spans="1:18">
       <c r="A47" t="s">
+        <v>506</v>
+      </c>
+      <c r="B47" t="s">
         <v>507</v>
       </c>
-      <c r="B47" t="s">
+      <c r="C47" t="s">
+        <v>50</v>
+      </c>
+      <c r="D47" t="s">
         <v>508</v>
       </c>
-      <c r="C47" t="s">
-        <v>15</v>
-      </c>
-      <c r="D47" t="s">
+      <c r="E47" t="s">
         <v>509</v>
       </c>
-      <c r="E47" t="s">
+      <c r="F47" t="s">
         <v>510</v>
       </c>
-      <c r="F47" t="s">
+      <c r="G47" s="2" t="s">
         <v>511</v>
       </c>
-      <c r="G47" s="2" t="s">
+      <c r="H47" t="s">
         <v>512</v>
       </c>
-      <c r="H47" t="s">
+      <c r="I47" t="s">
+        <v>512</v>
+      </c>
+      <c r="J47" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80524_milton keynes", ".\export_data\inspection_reports\80524_milton keynes")</f>
+        <v>0</v>
+      </c>
+      <c r="K47" t="s">
         <v>513</v>
       </c>
-      <c r="I47" t="s">
-        <v>513</v>
-      </c>
-      <c r="J47" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80418_norfolk", ".\export_data\inspection_reports\80418_norfolk")</f>
-        <v>0</v>
-      </c>
-      <c r="K47" t="s">
+      <c r="L47" t="s">
+        <v>9</v>
+      </c>
+      <c r="M47" t="s">
         <v>514</v>
-      </c>
-      <c r="L47" t="s">
-        <v>9</v>
-      </c>
-      <c r="M47" t="s">
-        <v>9</v>
       </c>
       <c r="N47" t="s">
         <v>515</v>
       </c>
       <c r="O47" t="s">
+        <v>9</v>
+      </c>
+      <c r="P47" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q47" t="s">
+        <v>82</v>
+      </c>
+      <c r="R47" t="s">
         <v>516</v>
-      </c>
-      <c r="P47" t="s">
-        <v>517</v>
-      </c>
-      <c r="Q47" t="s">
-        <v>12</v>
-      </c>
-      <c r="R47" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="48" spans="1:18">
       <c r="A48" t="s">
+        <v>517</v>
+      </c>
+      <c r="B48" t="s">
         <v>518</v>
       </c>
-      <c r="B48" t="s">
+      <c r="C48" t="s">
+        <v>15</v>
+      </c>
+      <c r="D48" t="s">
         <v>519</v>
       </c>
-      <c r="C48" t="s">
-        <v>2</v>
-      </c>
-      <c r="D48" t="s">
+      <c r="E48" t="s">
         <v>520</v>
       </c>
-      <c r="E48" t="s">
+      <c r="F48" t="s">
         <v>521</v>
       </c>
-      <c r="F48" t="s">
+      <c r="G48" s="2" t="s">
         <v>522</v>
       </c>
-      <c r="G48" s="2" t="s">
+      <c r="H48" t="s">
         <v>523</v>
       </c>
-      <c r="H48" t="s">
+      <c r="I48" t="s">
+        <v>523</v>
+      </c>
+      <c r="J48" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80418_norfolk", ".\export_data\inspection_reports\80418_norfolk")</f>
+        <v>0</v>
+      </c>
+      <c r="K48" t="s">
         <v>524</v>
       </c>
-      <c r="I48" t="s">
-        <v>524</v>
-      </c>
-      <c r="J48" s="3">
-        <f>HYPERLINK(".\.\export_data\inspection_reports\80530_north yorkshire", ".\export_data\inspection_reports\80530_north yorkshire")</f>
-        <v>0</v>
-      </c>
-      <c r="K48" t="s">
+      <c r="L48" t="s">
+        <v>9</v>
+      </c>
+      <c r="M48" t="s">
+        <v>9</v>
+      </c>
+      <c r="N48" t="s">
         <v>525</v>
       </c>
-      <c r="L48" t="s">
-        <v>9</v>
-      </c>
-      <c r="M48" t="s">
-        <v>9</v>
-      </c>
-      <c r="N48" t="s">
+      <c r="O48" t="s">
         <v>526</v>
       </c>
-      <c r="O48" t="s">
+      <c r="P48" t="s">
         <v>527</v>
-      </c>
-      <c r="P48" t="s">
-        <v>528</v>
       </c>
       <c r="Q48" t="s">
         <v>12</v>
@@ -4790,59 +4820,116 @@
     </row>
     <row r="49" spans="1:18">
       <c r="A49" t="s">
+        <v>528</v>
+      </c>
+      <c r="B49" t="s">
         <v>529</v>
       </c>
-      <c r="B49" t="s">
+      <c r="C49" t="s">
+        <v>2</v>
+      </c>
+      <c r="D49" t="s">
         <v>530</v>
       </c>
-      <c r="C49" t="s">
+      <c r="E49" t="s">
+        <v>531</v>
+      </c>
+      <c r="F49" t="s">
+        <v>532</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="H49" t="s">
+        <v>534</v>
+      </c>
+      <c r="I49" t="s">
+        <v>534</v>
+      </c>
+      <c r="J49" s="3">
+        <f>HYPERLINK(".\.\export_data\inspection_reports\80530_north yorkshire", ".\export_data\inspection_reports\80530_north yorkshire")</f>
+        <v>0</v>
+      </c>
+      <c r="K49" t="s">
+        <v>535</v>
+      </c>
+      <c r="L49" t="s">
+        <v>9</v>
+      </c>
+      <c r="M49" t="s">
+        <v>9</v>
+      </c>
+      <c r="N49" t="s">
+        <v>536</v>
+      </c>
+      <c r="O49" t="s">
+        <v>537</v>
+      </c>
+      <c r="P49" t="s">
+        <v>538</v>
+      </c>
+      <c r="Q49" t="s">
+        <v>12</v>
+      </c>
+      <c r="R49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:18">
+      <c r="A50" t="s">
+        <v>539</v>
+      </c>
+      <c r="B50" t="s">
+        <v>540</v>
+      </c>
+      <c r="C50" t="s">
         <v>185</v>
       </c>
-      <c r="D49" t="s">
-        <v>531</v>
-      </c>
-      <c r="E49" t="s">
-        <v>532</v>
-      </c>
-      <c r="F49" t="s">
-        <v>533</v>
-      </c>
-      <c r="G49" s="2" t="s">
-        <v>534</v>
-      </c>
-      <c r="H49" t="s">
-        <v>535</v>
-      </c>
-      <c r="I49" t="s">
-        <v>535</v>
-      </c>
-      <c r="J49" s="3">
+      <c r="D50" t="s">
+        <v>541</v>
+      </c>
+      <c r="E50" t="s">
+        <v>542</v>
+      </c>
+      <c r="F50" t="s">
+        <v>543</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="H50" t="s">
+        <v>545</v>
+      </c>
+      <c r="I50" t="s">
+        <v>545</v>
+      </c>
+      <c r="J50" s="3">
         <f>HYPERLINK(".\.\export_data\inspection_reports\80532_northumberland", ".\export_data\inspection_reports\80532_northumberland")</f>
         <v>0</v>
       </c>
-      <c r="K49" t="s">
-        <v>536</v>
-      </c>
-      <c r="L49" t="s">
-        <v>9</v>
-      </c>
-      <c r="M49" t="s">
-        <v>537</v>
-      </c>
-      <c r="N49" t="s">
-        <v>538</v>
-      </c>
-      <c r="O49" t="s">
-        <v>9</v>
-      </c>
-      <c r="P49" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q49" t="s">
+      <c r="K50" t="s">
+        <v>546</v>
+      </c>
+      <c r="L50" t="s">
+        <v>9</v>
+      </c>
+      <c r="M50" t="s">
+        <v>547</v>
+      </c>
+      <c r="N50" t="s">
+        <v>548</v>
+      </c>
+      <c r="O50" t="s">
+        <v>9</v>
+      </c>
+      <c r="P50" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q50" t="s">
         <v>82</v>
       </c>
-      <c r="R49" t="s">
-        <v>539</v>
+      <c r="R50" t="s">
+        <v>549</v>
       </c>
     </row>
   </sheetData>
@@ -4895,6 +4982,7 @@
     <hyperlink ref="G47" r:id="rId46"/>
     <hyperlink ref="G48" r:id="rId47"/>
     <hyperlink ref="G49" r:id="rId48"/>
+    <hyperlink ref="G50" r:id="rId49"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>